<commit_message>
New Merge runs app for HEM4
</commit_message>
<xml_diff>
--- a/resources/Target_Organ_Endpoints.xlsx
+++ b/resources/Target_Organ_Endpoints.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26501"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git_HEM4\HEM4\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/pfohl_marisa_epa_gov/Documents/Documents/Documents/OAR/Dose-Response Prioritization/OAQPS Toxicity Tables/HEM Dose-Response Library/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0B3BE12-31F4-45F3-8977-CBE6AB16E782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A8AAC33A-1D9E-4B8A-9E1D-186CE2A8E87C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28830" yWindow="1110" windowWidth="28770" windowHeight="15090" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Target Organ Endpoints" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Organ Endpoints'!$A$1:$P$303</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Organ Endpoints'!$A$1:$P$312</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Target Organ Endpoints'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="114210"/>
 </workbook>
@@ -1103,18 +1104,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1424,22 +1428,24 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P312"/>
-  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="41.5546875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="10.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="6.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.77734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="41.54296875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="6.81640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.81640625" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="8.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="9.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="8.77734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="8.26953125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.81640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.81640625" style="2" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.21875" style="2"/>
+    <col min="17" max="16384" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -1493,7 +1499,7 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="8" t="s">
         <v>245</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -3243,10 +3249,10 @@
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
+      <c r="A37" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="B37" s="6">
+      <c r="B37" s="7">
         <v>0</v>
       </c>
       <c r="C37" s="2">
@@ -5510,7 +5516,7 @@
       </c>
     </row>
     <row r="83" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A83" s="1" t="s">
+      <c r="A83" s="6" t="s">
         <v>318</v>
       </c>
       <c r="C83" s="2">
@@ -5848,7 +5854,7 @@
       </c>
     </row>
     <row r="90" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A90" s="2" t="s">
+      <c r="A90" s="8" t="s">
         <v>246</v>
       </c>
       <c r="B90" s="2" t="s">
@@ -6202,13 +6208,13 @@
         <v>20</v>
       </c>
       <c r="C97" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D97" s="2">
         <v>1</v>
       </c>
       <c r="E97" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F97" s="2">
         <v>0</v>
@@ -7480,7 +7486,7 @@
       </c>
     </row>
     <row r="123" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A123" s="1" t="s">
+      <c r="A123" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C123" s="2">
@@ -13592,7 +13598,7 @@
         <v>0</v>
       </c>
       <c r="G246" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H246" s="2">
         <v>0</v>
@@ -15825,10 +15831,10 @@
       </c>
     </row>
     <row r="292" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A292" s="1" t="s">
+      <c r="A292" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="B292" s="6">
+      <c r="B292" s="7">
         <v>0</v>
       </c>
       <c r="C292" s="2">
@@ -16425,7 +16431,7 @@
       </c>
     </row>
     <row r="304" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A304" s="2" t="s">
+      <c r="A304" s="9" t="s">
         <v>326</v>
       </c>
       <c r="C304" s="2">
@@ -16472,7 +16478,7 @@
       </c>
     </row>
     <row r="305" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A305" s="2" t="s">
+      <c r="A305" s="9" t="s">
         <v>327</v>
       </c>
       <c r="C305" s="2">
@@ -16519,7 +16525,7 @@
       </c>
     </row>
     <row r="306" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A306" s="2" t="s">
+      <c r="A306" s="9" t="s">
         <v>328</v>
       </c>
       <c r="C306" s="2">
@@ -16566,7 +16572,7 @@
       </c>
     </row>
     <row r="307" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A307" s="2" t="s">
+      <c r="A307" s="9" t="s">
         <v>329</v>
       </c>
       <c r="C307" s="2">
@@ -16613,7 +16619,7 @@
       </c>
     </row>
     <row r="308" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A308" s="2" t="s">
+      <c r="A308" s="9" t="s">
         <v>330</v>
       </c>
       <c r="C308" s="2">
@@ -16660,7 +16666,7 @@
       </c>
     </row>
     <row r="309" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A309" s="2" t="s">
+      <c r="A309" s="9" t="s">
         <v>331</v>
       </c>
       <c r="C309" s="2">
@@ -16707,7 +16713,7 @@
       </c>
     </row>
     <row r="310" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A310" s="2" t="s">
+      <c r="A310" s="9" t="s">
         <v>332</v>
       </c>
       <c r="C310" s="2">
@@ -16754,7 +16760,7 @@
       </c>
     </row>
     <row r="311" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A311" s="2" t="s">
+      <c r="A311" s="9" t="s">
         <v>333</v>
       </c>
       <c r="C311" s="2">
@@ -16801,7 +16807,7 @@
       </c>
     </row>
     <row r="312" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A312" s="2" t="s">
+      <c r="A312" s="9" t="s">
         <v>334</v>
       </c>
       <c r="C312" s="2">
@@ -16848,12 +16854,12 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P303" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:P312" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup scale="72" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
-    <oddFooter>&amp;LTarget Organ Endpoints&amp;C&amp;P&amp;RAugust 31, 2021</oddFooter>
+    <oddFooter>&amp;LTarget Organ Endpoints&amp;C&amp;P&amp;ROctober, 2025</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>